<commit_message>
Add Dethatching as a standalone service
- Workbook: new Dethatching tab using build_phase, 0.60 hr/1k sqft field
  labor + 1.00 hr mobilization, $75 dethatcher rental (Classen, 4-hr) as
  the only material. Tab inserted after Overseeding in tab order.
- Website services.html: new add-on card describing power-rake thatch
  removal, pairs with fall overseeding.
- Lead-form multi-select: "Dethatching (power-rake thatch removal)"
  option added on index.html and contact.html.
</commit_message>
<xml_diff>
--- a/pricing/Clean_and_Green_Pricing_Workbook.xlsx
+++ b/pricing/Clean_and_Green_Pricing_Workbook.xlsx
@@ -13,11 +13,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer Services" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprinkler Services" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overseeding" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 - Kill" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 - Prep" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 - Seed" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 4 - Establish" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Total" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dethatching" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 - Kill" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 - Prep" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 - Seed" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 4 - Establish" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Total" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="LawnSize">Assumptions!$B$3</definedName>
@@ -40,9 +41,11 @@
     <definedName name="AppMob">Assumptions!$B$20</definedName>
     <definedName name="OvsHrs">Assumptions!$B$21</definedName>
     <definedName name="OvsMob">Assumptions!$B$22</definedName>
-    <definedName name="SprAudHrs">Assumptions!$B$23</definedName>
-    <definedName name="SprHeadHrs">Assumptions!$B$24</definedName>
-    <definedName name="BHyveHrs">Assumptions!$B$25</definedName>
+    <definedName name="DethHrs">Assumptions!$B$23</definedName>
+    <definedName name="DethMob">Assumptions!$B$24</definedName>
+    <definedName name="SprAudHrs">Assumptions!$B$25</definedName>
+    <definedName name="SprHeadHrs">Assumptions!$B$26</definedName>
+    <definedName name="BHyveHrs">Assumptions!$B$27</definedName>
     <definedName name="Glyphosate">'Materials Catalog'!$I$3</definedName>
     <definedName name="Surfactant">'Materials Catalog'!$I$4</definedName>
     <definedName name="Tenacity">'Materials Catalog'!$I$5</definedName>
@@ -86,6 +89,9 @@
     <definedName name="OVE_Total">'Overseeding'!$F$24</definedName>
     <definedName name="OVE_Mat">'Overseeding'!$F16</definedName>
     <definedName name="OVE_Lab">'Overseeding'!$F22</definedName>
+    <definedName name="DET_Total">'Dethatching'!$F$19</definedName>
+    <definedName name="DET_Mat">'Dethatching'!$F11</definedName>
+    <definedName name="DET_Lab">'Dethatching'!$F17</definedName>
     <definedName name="GrandTotal">'Project Total'!$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1100,6 +1106,363 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Phase 3  |  Seed + Starter Fertilizer + Tenacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Scope of Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Apply starter fertilizer, then broadcast Valkyrie seed at 10 lb / 1,000 sq ft in two directions. Tank-mix Tenacity with non-ionic surfactant and apply at 0.18 oz / 1,000 sq ft for 21 days of pre-emergent weed protection. Top-dress lightly with peat moss to retain moisture, then begin the watering schedule (light 2-3x daily until germination).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Materials  (per 1,000 sq ft items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>$ / 1,000 sq ft</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t># Apps</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Cost (raw)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Cost (w/ markup)</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Starter fertilizer (24-25-4)</t>
+        </is>
+      </c>
+      <c r="C7" s="9">
+        <f>Starter</f>
+        <v/>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9">
+        <f>C7*D7*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>E7*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G7" s="26" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Valkyrie tall fescue seed</t>
+        </is>
+      </c>
+      <c r="C8" s="9">
+        <f>Seed</f>
+        <v/>
+      </c>
+      <c r="D8" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="9">
+        <f>C8*D8*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>E8*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G8" s="26" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Tenacity at-seeding pre-emergent</t>
+        </is>
+      </c>
+      <c r="C9" s="9">
+        <f>Tenacity</f>
+        <v/>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9">
+        <f>C9*D9*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>E9*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G9" s="26" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Non-Ionic Surfactant (Tenacity tank)</t>
+        </is>
+      </c>
+      <c r="C10" s="9">
+        <f>Surfactant</f>
+        <v/>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9">
+        <f>C10*D10*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>E10*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G10" s="26" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Peat moss top-dress</t>
+        </is>
+      </c>
+      <c r="C11" s="9">
+        <f>Peat</f>
+        <v/>
+      </c>
+      <c r="D11" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9">
+        <f>C11*D11*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="F11" s="10">
+        <f>E11*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G11" s="26" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>MATERIALS SUBTOTAL (with markup)</t>
+        </is>
+      </c>
+      <c r="E13" s="37">
+        <f>E7+E8+E9+E10+E11</f>
+        <v/>
+      </c>
+      <c r="F13" s="29">
+        <f>F7+F8+F9+F10+F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Hours basis</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Field labor (per 1,000 sq ft)</t>
+        </is>
+      </c>
+      <c r="C17" s="7">
+        <f>P3Hrs hr/1,000 sf</f>
+        <v/>
+      </c>
+      <c r="D17" s="38">
+        <f>P3Hrs*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="E17" s="9">
+        <f>LaborRate</f>
+        <v/>
+      </c>
+      <c r="F17" s="10">
+        <f>D17*E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="30" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Mobilization / setup</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Fixed hrs/job</t>
+        </is>
+      </c>
+      <c r="D18" s="38">
+        <f>P3Mob</f>
+        <v/>
+      </c>
+      <c r="E18" s="9">
+        <f>LaborRate</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>D18*E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="30" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>LABOR SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="F19" s="29">
+        <f>F17+F18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>PHASE 3  |  SEED + STARTER FERTILIZER + TENACITY - PHASE TOTAL</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="13">
+        <f>F13+F19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E7D32"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1398,7 +1761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B4D1F"/>
@@ -1606,7 +1969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2047,11 +2410,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler Audit Labor (flat)</t>
+          <t>Dethatching Labor (per 1,000 sq ft)</t>
         </is>
       </c>
       <c r="B23" s="22" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
@@ -2060,18 +2423,18 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Catch cup audit + diagnose + write DU report.</t>
+          <t>Power dethatch + rake/haul thatch debris.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler Repair Labor (per head)</t>
+          <t>Dethatching Mobilization Hours</t>
         </is>
       </c>
       <c r="B24" s="22" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
@@ -2080,25 +2443,65 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Replace a single sprinkler head incl. minor digging.</t>
+          <t>Equipment pickup/return + customer walk-through.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Sprinkler Audit Labor (flat)</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Catch cup audit + diagnose + write DU report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Sprinkler Repair Labor (per head)</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Replace a single sprinkler head incl. minor digging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>B-Hyve Smart Controller Install</t>
         </is>
       </c>
-      <c r="B25" s="22" t="n">
+      <c r="B27" s="22" t="n">
         <v>1.5</v>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>hours</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>FREE labor per Ryan's offer; baked into controller markup.</t>
         </is>
@@ -4686,6 +5089,304 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00A5D6A7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dethatching  |  Power-rake + thatch removal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Scope of Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Standalone power-dethatching service for thinning lawns with a thick thatch layer (typically &gt;1/2 inch). Power-rake removes built-up thatch so water, air, and nutrients can reach the soil. Crew hauls all debris. Most lawns only need this every 3-5 years; best paired with overseeding when scheduled in fall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Materials  (per 1,000 sq ft items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>$ / 1,000 sq ft</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t># Apps</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Cost (raw)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Cost (w/ markup)</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Materials  (per-job / one-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Cost each</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Cost (raw)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Cost (w/ markup)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Power dethatcher rental (4-hr)</t>
+        </is>
+      </c>
+      <c r="C9" s="9">
+        <f>Dethatcher</f>
+        <v/>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>E9*(1+Markup)</f>
+        <v/>
+      </c>
+      <c r="G9" s="26" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>MATERIALS SUBTOTAL (with markup)</t>
+        </is>
+      </c>
+      <c r="E11" s="37">
+        <f>E9</f>
+        <v/>
+      </c>
+      <c r="F11" s="29">
+        <f>F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Hours basis</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Field labor (per 1,000 sq ft)</t>
+        </is>
+      </c>
+      <c r="C15" s="7">
+        <f>DethHrs hr/1,000 sf</f>
+        <v/>
+      </c>
+      <c r="D15" s="38">
+        <f>DethHrs*(LawnSize/1000)</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>LaborRate</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>D15*E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="30" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Mobilization / setup</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Fixed hrs/job</t>
+        </is>
+      </c>
+      <c r="D16" s="38">
+        <f>DethMob</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>LaborRate</f>
+        <v/>
+      </c>
+      <c r="F16" s="10">
+        <f>D16*E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="30" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>LABOR SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="F17" s="29">
+        <f>F15+F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>DETHATCHING  |  POWER-RAKE + THATCH REMOVAL - PHASE TOTAL</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="13">
+        <f>F11+F17</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -5033,7 +5734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E7D32"/>
@@ -5355,361 +6056,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="002E7D32"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Phase 3  |  Seed + Starter Fertilizer + Tenacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Scope of Work</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Apply starter fertilizer, then broadcast Valkyrie seed at 10 lb / 1,000 sq ft in two directions. Tank-mix Tenacity with non-ionic surfactant and apply at 0.18 oz / 1,000 sq ft for 21 days of pre-emergent weed protection. Top-dress lightly with peat moss to retain moisture, then begin the watering schedule (light 2-3x daily until germination).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>Materials  (per 1,000 sq ft items)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>$ / 1,000 sq ft</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t># Apps</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Cost (raw)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Cost (w/ markup)</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Starter fertilizer (24-25-4)</t>
-        </is>
-      </c>
-      <c r="C7" s="9">
-        <f>Starter</f>
-        <v/>
-      </c>
-      <c r="D7" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="9">
-        <f>C7*D7*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="F7" s="10">
-        <f>E7*(1+Markup)</f>
-        <v/>
-      </c>
-      <c r="G7" s="26" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Valkyrie tall fescue seed</t>
-        </is>
-      </c>
-      <c r="C8" s="9">
-        <f>Seed</f>
-        <v/>
-      </c>
-      <c r="D8" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="9">
-        <f>C8*D8*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="F8" s="10">
-        <f>E8*(1+Markup)</f>
-        <v/>
-      </c>
-      <c r="G8" s="26" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Tenacity at-seeding pre-emergent</t>
-        </is>
-      </c>
-      <c r="C9" s="9">
-        <f>Tenacity</f>
-        <v/>
-      </c>
-      <c r="D9" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="9">
-        <f>C9*D9*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="F9" s="10">
-        <f>E9*(1+Markup)</f>
-        <v/>
-      </c>
-      <c r="G9" s="26" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Non-Ionic Surfactant (Tenacity tank)</t>
-        </is>
-      </c>
-      <c r="C10" s="9">
-        <f>Surfactant</f>
-        <v/>
-      </c>
-      <c r="D10" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="9">
-        <f>C10*D10*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="F10" s="10">
-        <f>E10*(1+Markup)</f>
-        <v/>
-      </c>
-      <c r="G10" s="26" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Peat moss top-dress</t>
-        </is>
-      </c>
-      <c r="C11" s="9">
-        <f>Peat</f>
-        <v/>
-      </c>
-      <c r="D11" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9">
-        <f>C11*D11*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="F11" s="10">
-        <f>E11*(1+Markup)</f>
-        <v/>
-      </c>
-      <c r="G11" s="26" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>MATERIALS SUBTOTAL (with markup)</t>
-        </is>
-      </c>
-      <c r="E13" s="37">
-        <f>E7+E8+E9+E10+E11</f>
-        <v/>
-      </c>
-      <c r="F13" s="29">
-        <f>F7+F8+F9+F10+F11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Hours basis</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Hours</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="n"/>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Field labor (per 1,000 sq ft)</t>
-        </is>
-      </c>
-      <c r="C17" s="7">
-        <f>P3Hrs hr/1,000 sf</f>
-        <v/>
-      </c>
-      <c r="D17" s="38">
-        <f>P3Hrs*(LawnSize/1000)</f>
-        <v/>
-      </c>
-      <c r="E17" s="9">
-        <f>LaborRate</f>
-        <v/>
-      </c>
-      <c r="F17" s="10">
-        <f>D17*E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="30" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="30" t="n"/>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Mobilization / setup</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Fixed hrs/job</t>
-        </is>
-      </c>
-      <c r="D18" s="38">
-        <f>P3Mob</f>
-        <v/>
-      </c>
-      <c r="E18" s="9">
-        <f>LaborRate</f>
-        <v/>
-      </c>
-      <c r="F18" s="10">
-        <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="30" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>LABOR SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="F19" s="29">
-        <f>F17+F18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="34" t="inlineStr">
-        <is>
-          <t>PHASE 3  |  SEED + STARTER FERTILIZER + TENACITY - PHASE TOTAL</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="13">
-        <f>F13+F19</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A5:G5"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>